<commit_message>
Solved saving and plotting bugs for behavior, olfa and audio
</commit_message>
<xml_diff>
--- a/soundstimuliFiles/defaultSoundConfig.xlsx
+++ b/soundstimuliFiles/defaultSoundConfig.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20410"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\homedir-cifs.nyumc.org\barrab01\Personal\Repos\PyBpodGUI\soundstimuliFiles\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rinberg Lab\Documents\pybpod3.11\PyBpodGUI\soundstimuliFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A2AA2C8-1DEF-4630-A6B6-0E7FE7D0D09C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="14025" xr2:uid="{C1995DA3-FBDC-4A92-B359-FA9BCCC23A57}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="14025"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="6">
   <si>
     <t>Freq</t>
   </si>
@@ -39,16 +38,16 @@
     <t>Duration</t>
   </si>
   <si>
-    <t>[1, 1.4, 1.9, 2.7, 3.7, 5.2, 7.2, 10]</t>
-  </si>
-  <si>
-    <t>[1, 1, 1, 1, 1, 1, 1, 1]</t>
+    <t>[0.1, 0.2, 0.5, 0.8, 1, 2, 5, 8]</t>
+  </si>
+  <si>
+    <t>[1,1,1,1,1,1,1,1]</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -393,12 +392,13 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E351CE68-72F0-43DC-AE65-5E699408626B}">
-  <dimension ref="A1:D3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="28.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -417,7 +417,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>10000</v>
+        <v>16000</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
@@ -426,20 +426,6 @@
         <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>16000</v>
-      </c>
-      <c r="B3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Small changes for behavior
</commit_message>
<xml_diff>
--- a/soundstimuliFiles/defaultSoundConfig.xlsx
+++ b/soundstimuliFiles/defaultSoundConfig.xlsx
@@ -38,10 +38,10 @@
     <t>Duration</t>
   </si>
   <si>
-    <t>[0.1, 0.2, 0.5, 0.8, 1, 2, 5, 8]</t>
-  </si>
-  <si>
     <t>[1,1,1,1,1,1,1,1]</t>
+  </si>
+  <si>
+    <t>[0.28, 0.33, 0.39, 0.46, 0.54, 0.64, 0.75, 0.9]</t>
   </si>
 </sst>
 </file>
@@ -77,8 +77,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -396,7 +399,7 @@
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="28.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="46.5703125" customWidth="1"/>
     <col min="3" max="3" width="17.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.5703125" bestFit="1" customWidth="1"/>
   </cols>
@@ -419,14 +422,14 @@
       <c r="A2">
         <v>16000</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" t="s">
-        <v>5</v>
-      </c>
       <c r="D2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Small modifications on rig E during behavior
</commit_message>
<xml_diff>
--- a/soundstimuliFiles/defaultSoundConfig.xlsx
+++ b/soundstimuliFiles/defaultSoundConfig.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="14025"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14340" windowHeight="4680"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>Freq</t>
   </si>
@@ -38,10 +38,13 @@
     <t>Duration</t>
   </si>
   <si>
+    <t>[0.28, 0.391, 0.54, 0.75, 1.05, 1.47, 2.04, 2.85]</t>
+  </si>
+  <si>
     <t>[1,1,1,1,1,1,1,1]</t>
   </si>
   <si>
-    <t>[0.28, 0.33, 0.39, 0.46, 0.54, 0.64, 0.75, 0.9]</t>
+    <t>[4,3,2,1,1,2,3,4]</t>
   </si>
 </sst>
 </file>
@@ -423,13 +426,13 @@
         <v>16000</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" t="s">
-        <v>4</v>
-      </c>
       <c r="D2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
adding modifications done in local on behavior rig E
</commit_message>
<xml_diff>
--- a/soundstimuliFiles/defaultSoundConfig.xlsx
+++ b/soundstimuliFiles/defaultSoundConfig.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="6">
   <si>
     <t>Freq</t>
   </si>
@@ -38,13 +38,10 @@
     <t>Duration</t>
   </si>
   <si>
-    <t>[0.28, 0.391, 0.54, 0.75, 1.05, 1.47, 2.04, 2.85]</t>
-  </si>
-  <si>
-    <t>[1,1,1,1,1,1,1,1]</t>
-  </si>
-  <si>
-    <t>[4,3,2,1,1,2,3,4]</t>
+    <t>[5, 8]</t>
+  </si>
+  <si>
+    <t>[1,1]</t>
   </si>
 </sst>
 </file>
@@ -80,11 +77,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -403,7 +397,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="46.5703125" customWidth="1"/>
-    <col min="3" max="3" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -425,14 +419,14 @@
       <c r="A2">
         <v>16000</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>4</v>
       </c>
       <c r="C2" t="s">
         <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>